<commit_message>
Alle LP + PV, aber Simu konvergiert nicht
</commit_message>
<xml_diff>
--- a/Stromnetze_Auslegungsdaten - Kopie.xlsx
+++ b/Stromnetze_Auslegungsdaten - Kopie.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Noah\Desktop\EE TH Köln\Semester 2\Stromnetze\Daten\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Stromnetze\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{389C58F9-916E-4819-A50E-1EB0C37C14D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AD3E630-7E2D-434B-BCE5-FFBE67646312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-132" yWindow="-132" windowWidth="23304" windowHeight="12504" xr2:uid="{BCB6E361-6B8C-4206-8358-FAA731AD6885}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{BCB6E361-6B8C-4206-8358-FAA731AD6885}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="46">
   <si>
     <t>Länge</t>
   </si>
@@ -162,6 +162,21 @@
   </si>
   <si>
     <t>Paralell</t>
+  </si>
+  <si>
+    <t>21.95</t>
+  </si>
+  <si>
+    <t>76.79</t>
+  </si>
+  <si>
+    <t>NAYY 4x35</t>
+  </si>
+  <si>
+    <t>BHS 27</t>
+  </si>
+  <si>
+    <t>BHS 27a</t>
   </si>
 </sst>
 </file>
@@ -210,7 +225,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -292,7 +307,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -608,14 +623,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{590A3F28-3505-4D03-AE8D-D666755562EE}">
-  <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -629,7 +644,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>10</v>
       </c>
@@ -644,35 +659,35 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>9</v>
-      </c>
-      <c r="B3">
-        <v>20</v>
+        <v>91</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>9</v>
-      </c>
-      <c r="B4">
-        <v>30</v>
+        <v>91</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>9</v>
       </c>
@@ -683,10 +698,10 @@
         <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>9</v>
       </c>
@@ -697,123 +712,123 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>20</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
       </c>
       <c r="D7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>30</v>
       </c>
       <c r="C8" t="s">
         <v>5</v>
       </c>
       <c r="D8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
         <v>6</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>6</v>
+      </c>
+      <c r="B11" t="s">
         <v>9</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C11" t="s">
         <v>10</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>5</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B12" s="1">
         <f>34.085+74.486</f>
         <v>108.571</v>
       </c>
-      <c r="C10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>4</v>
-      </c>
-      <c r="B11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>15</v>
-      </c>
       <c r="C12" t="s">
         <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>3</v>
-      </c>
-      <c r="B13">
-        <v>20</v>
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>3</v>
       </c>
-      <c r="B14">
-        <v>20</v>
+      <c r="B14" t="s">
+        <v>15</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>3</v>
       </c>
@@ -821,13 +836,13 @@
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D15" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>3</v>
       </c>
@@ -835,13 +850,13 @@
         <v>20</v>
       </c>
       <c r="C16" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D16" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>3</v>
       </c>
@@ -849,65 +864,93 @@
         <v>20</v>
       </c>
       <c r="C17" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>3</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18">
+        <v>20</v>
+      </c>
+      <c r="C18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>3</v>
+      </c>
+      <c r="B19">
+        <v>20</v>
+      </c>
+      <c r="C19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>3</v>
+      </c>
+      <c r="B20" t="s">
         <v>17</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C20" t="s">
         <v>12</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D20" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>2</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B21" t="s">
         <v>19</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C21" t="s">
         <v>18</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D21" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>2</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B22" t="s">
         <v>20</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C22" t="s">
         <v>18</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D22" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>1</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B23" t="s">
         <v>21</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C23" t="s">
         <v>12</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D23" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>